<commit_message>
Marketo TikToks Oct 30 + free-sheet paid offer
</commit_message>
<xml_diff>
--- a/free-budget-sheet/Paycheck-Budget-Starter-CalmColumnsCo.xlsx
+++ b/free-budget-sheet/Paycheck-Budget-Starter-CalmColumnsCo.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paycheck Budget" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upgrade" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paycheck Budget" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upgrade" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,11 +20,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="mmm d"/>
-    <numFmt numFmtId="166" formatCode="mmm d, yyyy"/>
+    <numFmt numFmtId="164" formatCode="mmm d, yyyy"/>
+    <numFmt numFmtId="165" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="mmm d"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -102,6 +103,18 @@
       <sz val="11"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="003F4F45"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -143,26 +156,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -192,6 +205,18 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -557,6 +582,93 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>Want the full system? Get the full planner on Etsy — 40% off launch sale through Nov 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>This free starter covers one paycheck. The paid CalmColumnsCo Google Sheets templates do more of the work. Sale price shown on Etsy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>Money Reset Mega Bundle (all 13 templates)</t>
+        </is>
+      </c>
+      <c r="B4" s="32" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/listing/4597077552?utm_source=freesheet&amp;utm_medium=landing</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="31" t="inlineStr">
+        <is>
+          <t>2027 Budget Planner</t>
+        </is>
+      </c>
+      <c r="B5" s="32" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/listing/4596462527?utm_source=freesheet&amp;utm_medium=landing</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t>Paycheck Budget template (both paychecks)</t>
+        </is>
+      </c>
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>https://www.etsy.com/listing/4597075314?utm_source=freesheet&amp;utm_medium=landing</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Your free budget is on the next tab: Paycheck Budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>A planning tool, not financial advice. CalmColumnsCo, c/o Mike Redler, 867 Boylston Street, 5th Floor #1586, Boston, MA 02116</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId3"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -627,7 +739,7 @@
           <t>Pay date</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
+      <c r="B5" s="33" t="n"/>
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="n"/>
@@ -636,7 +748,7 @@
           <t>Total income</t>
         </is>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="34">
         <f>B8</f>
         <v/>
       </c>
@@ -647,10 +759,10 @@
           <t>Take-home pay</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="35" t="n">
         <v>1800</v>
       </c>
-      <c r="C6" s="9" t="n"/>
+      <c r="C6" s="36" t="n"/>
       <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="n"/>
       <c r="F6" s="6" t="inlineStr">
@@ -658,7 +770,7 @@
           <t>Fixed bills</t>
         </is>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="34">
         <f>C20</f>
         <v/>
       </c>
@@ -669,10 +781,10 @@
           <t>Other income</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="35" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="9" t="n"/>
+      <c r="C7" s="36" t="n"/>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="n"/>
       <c r="F7" s="6" t="inlineStr">
@@ -680,7 +792,7 @@
           <t>Savings &amp; debt</t>
         </is>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="34">
         <f>C27</f>
         <v/>
       </c>
@@ -691,11 +803,11 @@
           <t>Total income</t>
         </is>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="37">
         <f>B6+B7</f>
         <v/>
       </c>
-      <c r="C8" s="9" t="n"/>
+      <c r="C8" s="36" t="n"/>
       <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="6" t="inlineStr">
@@ -703,15 +815,15 @@
           <t>Everyday spending</t>
         </is>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="34">
         <f>C34</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n"/>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
+      <c r="B9" s="36" t="n"/>
+      <c r="C9" s="36" t="n"/>
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="12" t="inlineStr">
@@ -719,7 +831,7 @@
           <t>Leftover</t>
         </is>
       </c>
-      <c r="G9" s="13">
+      <c r="G9" s="38">
         <f>G5-G6-G7-G8</f>
         <v/>
       </c>
@@ -730,8 +842,8 @@
           <t>FIXED BILLS</t>
         </is>
       </c>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="14" t="n"/>
+      <c r="B10" s="39" t="n"/>
+      <c r="C10" s="39" t="n"/>
       <c r="D10" s="4" t="n"/>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="12" t="inlineStr">
@@ -750,12 +862,12 @@
           <t>Bill</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="40" t="inlineStr">
         <is>
           <t>Due date</t>
         </is>
       </c>
-      <c r="C11" s="16" t="inlineStr">
+      <c r="C11" s="40" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
@@ -775,8 +887,8 @@
           <t>Rent / mortgage</t>
         </is>
       </c>
-      <c r="B12" s="18" t="n"/>
-      <c r="C12" s="8" t="n">
+      <c r="B12" s="41" t="n"/>
+      <c r="C12" s="35" t="n">
         <v>950</v>
       </c>
       <c r="D12" s="17" t="inlineStr">
@@ -794,8 +906,8 @@
           <t>Phone</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n"/>
-      <c r="C13" s="8" t="n">
+      <c r="B13" s="41" t="n"/>
+      <c r="C13" s="35" t="n">
         <v>45</v>
       </c>
       <c r="D13" s="17" t="inlineStr">
@@ -813,8 +925,8 @@
           <t>Internet</t>
         </is>
       </c>
-      <c r="B14" s="18" t="n"/>
-      <c r="C14" s="8" t="n">
+      <c r="B14" s="41" t="n"/>
+      <c r="C14" s="35" t="n">
         <v>60</v>
       </c>
       <c r="D14" s="17" t="inlineStr">
@@ -832,8 +944,8 @@
           <t>Car payment</t>
         </is>
       </c>
-      <c r="B15" s="18" t="n"/>
-      <c r="C15" s="8" t="n">
+      <c r="B15" s="41" t="n"/>
+      <c r="C15" s="35" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="17" t="inlineStr">
@@ -851,8 +963,8 @@
           <t>Insurance</t>
         </is>
       </c>
-      <c r="B16" s="18" t="n"/>
-      <c r="C16" s="8" t="n">
+      <c r="B16" s="41" t="n"/>
+      <c r="C16" s="35" t="n">
         <v>120</v>
       </c>
       <c r="D16" s="17" t="inlineStr">
@@ -870,8 +982,8 @@
           <t>Utilities</t>
         </is>
       </c>
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="8" t="n">
+      <c r="B17" s="41" t="n"/>
+      <c r="C17" s="35" t="n">
         <v>90</v>
       </c>
       <c r="D17" s="17" t="inlineStr">
@@ -889,8 +1001,8 @@
           <t>Subscriptions</t>
         </is>
       </c>
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="8" t="n">
+      <c r="B18" s="41" t="n"/>
+      <c r="C18" s="35" t="n">
         <v>25</v>
       </c>
       <c r="D18" s="17" t="inlineStr">
@@ -904,8 +1016,8 @@
     </row>
     <row r="19">
       <c r="A19" s="17" t="n"/>
-      <c r="B19" s="18" t="n"/>
-      <c r="C19" s="8" t="n"/>
+      <c r="B19" s="41" t="n"/>
+      <c r="C19" s="35" t="n"/>
       <c r="D19" s="17" t="n"/>
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="n"/>
@@ -917,8 +1029,8 @@
           <t>Total bills</t>
         </is>
       </c>
-      <c r="B20" s="9" t="n"/>
-      <c r="C20" s="11">
+      <c r="B20" s="36" t="n"/>
+      <c r="C20" s="37">
         <f>SUM(C12:C19)</f>
         <v/>
       </c>
@@ -932,8 +1044,8 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n"/>
-      <c r="B21" s="9" t="n"/>
-      <c r="C21" s="9" t="n"/>
+      <c r="B21" s="36" t="n"/>
+      <c r="C21" s="36" t="n"/>
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="n"/>
       <c r="F21" s="2" t="n"/>
@@ -945,8 +1057,8 @@
           <t>SAVINGS &amp; DEBT</t>
         </is>
       </c>
-      <c r="B22" s="14" t="n"/>
-      <c r="C22" s="14" t="n"/>
+      <c r="B22" s="39" t="n"/>
+      <c r="C22" s="39" t="n"/>
       <c r="D22" s="4" t="n"/>
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="n"/>
@@ -958,8 +1070,8 @@
           <t>Goal</t>
         </is>
       </c>
-      <c r="B23" s="16" t="n"/>
-      <c r="C23" s="16" t="inlineStr">
+      <c r="B23" s="40" t="n"/>
+      <c r="C23" s="40" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
@@ -975,8 +1087,8 @@
           <t>Emergency fund</t>
         </is>
       </c>
-      <c r="B24" s="8" t="n"/>
-      <c r="C24" s="8" t="n">
+      <c r="B24" s="35" t="n"/>
+      <c r="C24" s="35" t="n">
         <v>100</v>
       </c>
       <c r="D24" s="2" t="n"/>
@@ -990,8 +1102,8 @@
           <t>Extra debt payment</t>
         </is>
       </c>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="8" t="n">
+      <c r="B25" s="35" t="n"/>
+      <c r="C25" s="35" t="n">
         <v>50</v>
       </c>
       <c r="D25" s="2" t="n"/>
@@ -1001,8 +1113,8 @@
     </row>
     <row r="26">
       <c r="A26" s="17" t="n"/>
-      <c r="B26" s="8" t="n"/>
-      <c r="C26" s="8" t="n"/>
+      <c r="B26" s="35" t="n"/>
+      <c r="C26" s="35" t="n"/>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="n"/>
@@ -1014,8 +1126,8 @@
           <t>Total savings &amp; debt</t>
         </is>
       </c>
-      <c r="B27" s="9" t="n"/>
-      <c r="C27" s="11">
+      <c r="B27" s="36" t="n"/>
+      <c r="C27" s="37">
         <f>SUM(C24:C26)</f>
         <v/>
       </c>
@@ -1026,8 +1138,8 @@
     </row>
     <row r="28">
       <c r="A28" s="2" t="n"/>
-      <c r="B28" s="9" t="n"/>
-      <c r="C28" s="9" t="n"/>
+      <c r="B28" s="36" t="n"/>
+      <c r="C28" s="36" t="n"/>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="n"/>
@@ -1039,8 +1151,8 @@
           <t>EVERYDAY SPENDING</t>
         </is>
       </c>
-      <c r="B29" s="14" t="n"/>
-      <c r="C29" s="14" t="n"/>
+      <c r="B29" s="39" t="n"/>
+      <c r="C29" s="39" t="n"/>
       <c r="D29" s="4" t="n"/>
       <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="n"/>
@@ -1052,8 +1164,8 @@
           <t>Category</t>
         </is>
       </c>
-      <c r="B30" s="16" t="n"/>
-      <c r="C30" s="16" t="inlineStr">
+      <c r="B30" s="40" t="n"/>
+      <c r="C30" s="40" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
@@ -1069,8 +1181,8 @@
           <t>Groceries</t>
         </is>
       </c>
-      <c r="B31" s="8" t="n"/>
-      <c r="C31" s="8" t="n">
+      <c r="B31" s="35" t="n"/>
+      <c r="C31" s="35" t="n">
         <v>200</v>
       </c>
       <c r="D31" s="2" t="n"/>
@@ -1084,8 +1196,8 @@
           <t>Gas / transit</t>
         </is>
       </c>
-      <c r="B32" s="8" t="n"/>
-      <c r="C32" s="8" t="n">
+      <c r="B32" s="35" t="n"/>
+      <c r="C32" s="35" t="n">
         <v>80</v>
       </c>
       <c r="D32" s="2" t="n"/>
@@ -1099,8 +1211,8 @@
           <t>Fun money</t>
         </is>
       </c>
-      <c r="B33" s="8" t="n"/>
-      <c r="C33" s="8" t="n">
+      <c r="B33" s="35" t="n"/>
+      <c r="C33" s="35" t="n">
         <v>50</v>
       </c>
       <c r="D33" s="2" t="n"/>
@@ -1114,8 +1226,8 @@
           <t>Total everyday spending</t>
         </is>
       </c>
-      <c r="B34" s="9" t="n"/>
-      <c r="C34" s="11">
+      <c r="B34" s="36" t="n"/>
+      <c r="C34" s="37">
         <f>SUM(C31:C33)</f>
         <v/>
       </c>
@@ -1198,7 +1310,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1304,7 +1416,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>